<commit_message>
Corrida | SFE-VTS | 2026-05-27 10:46:42.71737
</commit_message>
<xml_diff>
--- a/indicadores/SFE-VTS_out.xlsx
+++ b/indicadores/SFE-VTS_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">26/05/2026</t>
+    <t xml:space="preserve">27/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2048,7 +2048,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.480193712861889</v>
+        <v>0.478481700729284</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2106,7 +2106,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.188771332285967</v>
+        <v>0.189502960822115</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2176,7 +2176,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0488987877230635</v>
+        <v>0.0487345748793635</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2206,7 +2206,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0015423858555931</v>
+        <v>0.00160090953171806</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -24707,7 +24707,7 @@
         <v>481</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0190359254144888</v>
+        <v>-0.0185568330535138</v>
       </c>
     </row>
     <row r="6">
@@ -24715,7 +24715,7 @@
         <v>482</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.000220415999674493</v>
+        <v>0.00061200369648616</v>
       </c>
     </row>
     <row r="7">
@@ -24723,7 +24723,7 @@
         <v>483</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0195245017412651</v>
+        <v>0.0209696713615437</v>
       </c>
     </row>
     <row r="8">
@@ -24731,7 +24731,7 @@
         <v>484</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0584296664443222</v>
+        <v>0.0598954505221596</v>
       </c>
     </row>
     <row r="9">
@@ -24739,7 +24739,7 @@
         <v>485</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.0837319531598721</v>
+        <v>0.0851178356036261</v>
       </c>
     </row>
     <row r="10">
@@ -24747,7 +24747,7 @@
         <v>486</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.109439412489627</v>
+        <v>0.110714179512468</v>
       </c>
     </row>
     <row r="11">
@@ -24755,7 +24755,7 @@
         <v>487</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.169161740460132</v>
+        <v>0.169762164206358</v>
       </c>
     </row>
     <row r="12">
@@ -24763,7 +24763,7 @@
         <v>488</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.241588881646484</v>
+        <v>0.24185920879637</v>
       </c>
     </row>
     <row r="13">
@@ -24771,7 +24771,7 @@
         <v>489</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.331304291695584</v>
+        <v>0.3320134621667</v>
       </c>
     </row>
     <row r="14">
@@ -24779,7 +24779,7 @@
         <v>490</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.434478229933293</v>
+        <v>0.435319377953837</v>
       </c>
     </row>
     <row r="15">
@@ -24787,7 +24787,7 @@
         <v>491</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.470290489502907</v>
+        <v>0.470778581408282</v>
       </c>
     </row>
     <row r="16">
@@ -24795,7 +24795,7 @@
         <v>492</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.461830464357797</v>
+        <v>0.461655478973808</v>
       </c>
     </row>
     <row r="17">
@@ -24803,7 +24803,7 @@
         <v>493</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.472530538173138</v>
+        <v>0.471332904617273</v>
       </c>
     </row>
     <row r="18">
@@ -24811,7 +24811,7 @@
         <v>494</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.480193712861889</v>
+        <v>0.478481700729284</v>
       </c>
     </row>
     <row r="19">
@@ -24819,7 +24819,7 @@
         <v>495</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.474966912863999</v>
+        <v>0.473767582855067</v>
       </c>
     </row>
     <row r="20">
@@ -24827,7 +24827,7 @@
         <v>496</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.453529153211174</v>
+        <v>0.453598143044007</v>
       </c>
     </row>
     <row r="21">
@@ -24835,7 +24835,7 @@
         <v>497</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.424297829806344</v>
+        <v>0.425370518017448</v>
       </c>
     </row>
     <row r="22">
@@ -24843,7 +24843,7 @@
         <v>498</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.414498522633324</v>
+        <v>0.416001426370137</v>
       </c>
     </row>
     <row r="23">
@@ -24851,7 +24851,7 @@
         <v>499</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.380754761594</v>
+        <v>0.382630418645754</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-VTS | 2026-06-17 12:11:19.541223
</commit_message>
<xml_diff>
--- a/indicadores/SFE-VTS_out.xlsx
+++ b/indicadores/SFE-VTS_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="502">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Ventas en supermercados de gran superficie en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Ventas en supermercados de gran superficie</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">td</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,7 +113,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">27/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2016,9 +2022,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2029,7 +2039,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2043,12 +2053,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.478481700729284</v>
+        <v>0.478830125154761</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2059,7 +2069,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2087,7 +2097,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2101,12 +2111,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.189502960822115</v>
+        <v>0.188095730059492</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2129,7 +2139,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2143,7 +2153,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2157,7 +2167,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2171,12 +2181,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0487345748793635</v>
+        <v>0.0486495308163639</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2187,7 +2197,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2201,12 +2211,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00160090953171806</v>
+        <v>0.00162431521024957</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2349,10 +2359,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2365,10 +2375,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2392,66 +2402,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>33.4797059254454</v>
@@ -2504,7 +2514,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>33.3060083378816</v>
@@ -2561,7 +2571,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>37.9692987947347</v>
@@ -2618,7 +2628,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>35.713541991153</v>
@@ -2675,7 +2685,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>37.5980903286665</v>
@@ -2732,7 +2742,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>36.9439307123721</v>
@@ -2789,7 +2799,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>37.6693905023669</v>
@@ -2846,7 +2856,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>38.978862142858</v>
@@ -2903,7 +2913,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>34.3132257663153</v>
@@ -2960,7 +2970,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>37.9146222854368</v>
@@ -3017,7 +3027,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>40.6877505181205</v>
@@ -3074,7 +3084,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>53.0934076501108</v>
@@ -3131,7 +3141,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>38.0009795058602</v>
@@ -3190,7 +3200,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>38.6242813955135</v>
@@ -3249,7 +3259,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>44.305796201468</v>
@@ -3308,7 +3318,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>40.0119114284569</v>
@@ -3367,7 +3377,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>41.8193697920289</v>
@@ -3426,7 +3436,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>40.2862499571217</v>
@@ -3485,7 +3495,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>42.6126070318909</v>
@@ -3544,7 +3554,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>43.7183359620312</v>
@@ -3603,7 +3613,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>40.0703428489697</v>
@@ -3662,7 +3672,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>45.2124778162883</v>
@@ -3721,7 +3731,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>42.9176572777108</v>
@@ -3780,7 +3790,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>56.1786328511873</v>
@@ -3839,7 +3849,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>40.6564200140089</v>
@@ -3898,7 +3908,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>40.6180510688295</v>
@@ -3957,7 +3967,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>45.975874794518</v>
@@ -4016,7 +4026,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>43.5202149614007</v>
@@ -4075,7 +4085,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>44.0782508940967</v>
@@ -4134,7 +4144,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>43.1142291535354</v>
@@ -4193,7 +4203,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>47.4662428787248</v>
@@ -4252,7 +4262,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>44.3532803363395</v>
@@ -4311,7 +4321,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>41.8107595419136</v>
@@ -4370,7 +4380,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>47.3936382195398</v>
@@ -4429,7 +4439,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>42.8544047774805</v>
@@ -4488,7 +4498,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>57.5487161052578</v>
@@ -4547,7 +4557,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>42.8460509569636</v>
@@ -4606,7 +4616,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>44.6237338981167</v>
@@ -4665,7 +4675,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>47.8859340583714</v>
@@ -4724,7 +4734,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>55.2055708998175</v>
@@ -4783,7 +4793,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>49.5101943831275</v>
@@ -4842,7 +4852,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>51.1238957201712</v>
@@ -4901,7 +4911,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>55.7326836743868</v>
@@ -4960,7 +4970,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>54.4617861487881</v>
@@ -5019,7 +5029,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>53.7325397195214</v>
@@ -5078,7 +5088,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>54.7850961270526</v>
@@ -5137,7 +5147,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>52.6775538579446</v>
@@ -5196,7 +5206,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>72.1868974586626</v>
@@ -5255,7 +5265,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>49.8632856469193</v>
@@ -5314,7 +5324,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>49.5524526271847</v>
@@ -5373,7 +5383,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>56.7500057263969</v>
@@ -5432,7 +5442,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>54.9077889492995</v>
@@ -5491,7 +5501,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>48.9056929463264</v>
@@ -5550,7 +5560,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>53.9477405904492</v>
@@ -5609,7 +5619,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>54.3198077381164</v>
@@ -5668,7 +5678,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>51.2192802592236</v>
@@ -5727,7 +5737,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>49.8473901012916</v>
@@ -5786,7 +5796,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>49.9932241419395</v>
@@ -5845,7 +5855,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>48.5632980291665</v>
@@ -5904,7 +5914,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>63.4995574920066</v>
@@ -5963,7 +5973,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>47.8401418462867</v>
@@ -6022,7 +6032,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>46.3013463915496</v>
@@ -6081,7 +6091,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>51.5935642539138</v>
@@ -6140,7 +6150,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>41.518924012</v>
@@ -6199,7 +6209,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>38.3833455811925</v>
@@ -6258,7 +6268,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>40.3682585013639</v>
@@ -6317,7 +6327,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>37.7715773488491</v>
@@ -6376,7 +6386,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>35.9475349264465</v>
@@ -6435,7 +6445,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>33.7911899749565</v>
@@ -6494,7 +6504,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>34.7649788344969</v>
@@ -6553,7 +6563,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>34.5718294507559</v>
@@ -6612,7 +6622,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>44.8805786639615</v>
@@ -6671,7 +6681,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>31.109198246246</v>
@@ -6730,7 +6740,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>31.0573931334302</v>
@@ -6789,7 +6799,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>35.6970933821698</v>
@@ -6848,7 +6858,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>32.8966260536843</v>
@@ -6907,7 +6917,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>34.9175290710097</v>
@@ -6966,7 +6976,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>35.4777556293598</v>
@@ -7025,7 +7035,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>36.3153578704702</v>
@@ -7084,7 +7094,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>37.744308670855</v>
@@ -7143,7 +7153,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>36.0014728223688</v>
@@ -7202,7 +7212,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>38.0827660832347</v>
@@ -7261,7 +7271,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>37.4487146694544</v>
@@ -7320,7 +7330,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>48.3380578735251</v>
@@ -7379,7 +7389,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>36.0943988938968</v>
@@ -7438,7 +7448,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>36.4621985984889</v>
@@ -7497,7 +7507,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>38.7336104276033</v>
@@ -7556,7 +7566,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>39.4138518837729</v>
@@ -7615,7 +7625,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>39.9674090585143</v>
@@ -7674,7 +7684,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>37.6136876202489</v>
@@ -7733,7 +7743,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>39.7784037274606</v>
@@ -7792,7 +7802,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>38.806054886697</v>
@@ -7851,7 +7861,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>36.2750532282361</v>
@@ -7910,7 +7920,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>43.6059860871923</v>
@@ -7969,7 +7979,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>40.062055261304</v>
@@ -8028,7 +8038,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>56.9144530034368</v>
@@ -8087,7 +8097,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>41.2746337165111</v>
@@ -8146,7 +8156,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>38.8511943286517</v>
@@ -8205,7 +8215,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>43.0269742500609</v>
@@ -8264,7 +8274,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>43.1492508459908</v>
@@ -8323,7 +8333,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>42.825655989799</v>
@@ -8382,7 +8392,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>41.7962366538369</v>
@@ -8441,7 +8451,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>45.915426764125</v>
@@ -8500,7 +8510,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>42.2578770299887</v>
@@ -8559,7 +8569,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>40.840691260433</v>
@@ -8618,7 +8628,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>46.0828566267568</v>
@@ -8677,7 +8687,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>42.8720004322264</v>
@@ -8736,7 +8746,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>55.9196912510207</v>
@@ -8795,7 +8805,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>42.7699163229834</v>
@@ -8854,7 +8864,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>42.5523993146961</v>
@@ -8913,7 +8923,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>46.2481077123028</v>
@@ -8972,7 +8982,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>48.7278613835288</v>
@@ -9031,7 +9041,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>46.1904087567981</v>
@@ -9090,7 +9100,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>47.5455559887532</v>
@@ -9149,7 +9159,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>50.7791925874483</v>
@@ -9208,7 +9218,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>48.8670551517541</v>
@@ -9267,7 +9277,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>48.5709526477012</v>
@@ -9326,7 +9336,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>50.4703037808867</v>
@@ -9385,7 +9395,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>49.7657994467289</v>
@@ -9444,7 +9454,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>67.8471924955045</v>
@@ -9503,7 +9513,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>49.4910750392825</v>
@@ -9562,7 +9572,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>47.0598460106241</v>
@@ -9621,7 +9631,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>54.9523830392864</v>
@@ -9680,7 +9690,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>54.1028163609708</v>
@@ -9739,7 +9749,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>52.962332522042</v>
@@ -9798,7 +9808,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>57.556723067928</v>
@@ -9857,7 +9867,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>58.7468076591782</v>
@@ -9916,7 +9926,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>59.4634016518974</v>
@@ -9975,7 +9985,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>58.9147247388693</v>
@@ -10034,7 +10044,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>60.1888910063108</v>
@@ -10093,7 +10103,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>60.5500235337906</v>
@@ -10152,7 +10162,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>78.8388012261361</v>
@@ -10211,7 +10221,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>59.8722788688506</v>
@@ -10270,7 +10280,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>59.225920283722</v>
@@ -10329,7 +10339,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>66.1541383307824</v>
@@ -10388,7 +10398,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>59.3234191162563</v>
@@ -10447,7 +10457,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>61.6533832329143</v>
@@ -10506,7 +10516,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>61.0069476157406</v>
@@ -10565,7 +10575,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>61.0952096147454</v>
@@ -10624,7 +10634,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>64.850396525213</v>
@@ -10683,7 +10693,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>59.1491638816969</v>
@@ -10742,7 +10752,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>63.1556867776562</v>
@@ -10801,7 +10811,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>63.312853480464</v>
@@ -10860,7 +10870,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>78.6360916795225</v>
@@ -10919,7 +10929,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>59.1449661445191</v>
@@ -10978,7 +10988,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>54.7056687099305</v>
@@ -11037,7 +11047,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>59.2497699358939</v>
@@ -11096,7 +11106,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>59.3013631365914</v>
@@ -11155,7 +11165,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>61.1140351498426</v>
@@ -11214,7 +11224,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>60.0158727145587</v>
@@ -11273,7 +11283,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>62.9986371584144</v>
@@ -11332,7 +11342,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>62.5251129321855</v>
@@ -11391,7 +11401,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>57.2055967024982</v>
@@ -11450,7 +11460,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>62.5831088242198</v>
@@ -11509,7 +11519,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>61.6532455371085</v>
@@ -11568,7 +11578,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>77.2774635524026</v>
@@ -11627,7 +11637,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>60.5458024301745</v>
@@ -11686,7 +11696,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>56.8184583031682</v>
@@ -11745,7 +11755,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>62.0141682105783</v>
@@ -11804,7 +11814,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>61.7398957430712</v>
@@ -11863,7 +11873,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>65.6179202340739</v>
@@ -11922,7 +11932,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>64.1607750988433</v>
@@ -11981,7 +11991,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>67.916300726943</v>
@@ -12040,7 +12050,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>64.5329491201723</v>
@@ -12099,7 +12109,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>62.4062549480407</v>
@@ -12158,7 +12168,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>66.8065677520202</v>
@@ -12217,7 +12227,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>63.115570227965</v>
@@ -12276,7 +12286,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>83.7085066355761</v>
@@ -12335,7 +12345,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>62.6103504491318</v>
@@ -12394,7 +12404,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>59.9342721201833</v>
@@ -12453,7 +12463,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>66.9507067127561</v>
@@ -12512,7 +12522,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>67.6899651604716</v>
@@ -12571,7 +12581,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>64.9005951878246</v>
@@ -12630,7 +12640,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>67.5304450196394</v>
@@ -12689,7 +12699,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>71.8215010906229</v>
@@ -12748,7 +12758,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>68.4988568223483</v>
@@ -12807,7 +12817,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>65.4350249278905</v>
@@ -12866,7 +12876,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>70.9296618196991</v>
@@ -12925,7 +12935,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>68.708559634352</v>
@@ -12984,7 +12994,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>84.3861202939591</v>
@@ -13043,7 +13053,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>67.3418290761161</v>
@@ -13102,7 +13112,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>66.0805552440405</v>
@@ -13161,7 +13171,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>69.1595347748823</v>
@@ -13220,7 +13230,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>69.664565003026</v>
@@ -13279,7 +13289,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>65.1293589434952</v>
@@ -13338,7 +13348,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>69.6530772983895</v>
@@ -13397,7 +13407,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>70.1608831251035</v>
@@ -13456,7 +13466,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>69.3746128211922</v>
@@ -13515,7 +13525,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>67.5126361684527</v>
@@ -13574,7 +13584,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>68.4617667474369</v>
@@ -13633,7 +13643,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>68.2304806898315</v>
@@ -13692,7 +13702,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>84.287891303543</v>
@@ -13751,7 +13761,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>65.7198131456301</v>
@@ -13810,7 +13820,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>63.6117105326874</v>
@@ -13869,7 +13879,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>68.9198254492483</v>
@@ -13928,7 +13938,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>63.8281156742387</v>
@@ -13987,7 +13997,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>65.7925589813796</v>
@@ -14046,7 +14056,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>71.0131976773351</v>
@@ -14105,7 +14115,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>69.7118816298077</v>
@@ -14164,7 +14174,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>71.037834435853</v>
@@ -14223,7 +14233,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>65.6668007008888</v>
@@ -14282,7 +14292,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>68.5183145312456</v>
@@ -14341,7 +14351,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>70.6486028546507</v>
@@ -14400,7 +14410,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>87.6755302079907</v>
@@ -14459,7 +14469,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>69.4751740511263</v>
@@ -14518,7 +14528,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>61.5910160002752</v>
@@ -14577,7 +14587,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>68.8223655699816</v>
@@ -14636,7 +14646,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>66.7665785934393</v>
@@ -14695,7 +14705,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>69.4113274541812</v>
@@ -14754,7 +14764,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>68.1285504218711</v>
@@ -14813,7 +14823,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>67.4089802092139</v>
@@ -14872,7 +14882,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>68.9909319522751</v>
@@ -14931,7 +14941,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>62.0467321549659</v>
@@ -14990,7 +15000,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>68.8912021128404</v>
@@ -15049,7 +15059,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>71.0019111671171</v>
@@ -15108,7 +15118,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>83.0914056197421</v>
@@ -15167,7 +15177,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>66.3939310116625</v>
@@ -15226,7 +15236,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>62.0033712676267</v>
@@ -15285,7 +15295,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>64.6191464932838</v>
@@ -15344,7 +15354,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>63.0571954776011</v>
@@ -15403,7 +15413,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>65.5068976312164</v>
@@ -15462,7 +15472,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>65.8667596957587</v>
@@ -15521,7 +15531,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>68.2946855408191</v>
@@ -15580,7 +15590,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>68.0302202263947</v>
@@ -15639,7 +15649,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>60.3564097091595</v>
@@ -15698,7 +15708,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>67.5326763956336</v>
@@ -15757,7 +15767,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>69.3073778107288</v>
@@ -15816,7 +15826,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>83.9100542585407</v>
@@ -15875,7 +15885,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>64.3723638387911</v>
@@ -15934,7 +15944,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>59.7859532066719</v>
@@ -15993,7 +16003,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>61.9712747282311</v>
@@ -16052,7 +16062,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>58.4624234231622</v>
@@ -16111,7 +16121,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>59.1888666887085</v>
@@ -16170,7 +16180,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>58.3457816304821</v>
@@ -16229,7 +16239,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>58.7077752248538</v>
@@ -16288,7 +16298,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>57.2428142938148</v>
@@ -16347,7 +16357,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>54.3862264618812</v>
@@ -16406,7 +16416,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>56.2061908579481</v>
@@ -16465,7 +16475,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>57.4673778341718</v>
@@ -16524,7 +16534,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>71.7876594576435</v>
@@ -16583,7 +16593,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>58.3231930737046</v>
@@ -16642,7 +16652,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>52.9789996313081</v>
@@ -16701,7 +16711,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>56.6096443344943</v>
@@ -16760,7 +16770,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>58.101757049239</v>
@@ -16819,7 +16829,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>56.2488574008204</v>
@@ -16878,7 +16888,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>54.8430358457557</v>
@@ -16937,7 +16947,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>57.3056874976336</v>
@@ -16996,7 +17006,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>58.1816013936552</v>
@@ -17055,7 +17065,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>55.2999567096437</v>
@@ -17114,7 +17124,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>57.0322791288457</v>
@@ -17173,7 +17183,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>58.7057118543298</v>
@@ -17232,7 +17242,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>72.9715325603057</v>
@@ -17291,7 +17301,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>56.0086774906495</v>
@@ -17350,7 +17360,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>53.3194944007524</v>
@@ -17409,7 +17419,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>60.9345718217467</v>
@@ -17468,7 +17478,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>55.9824120593804</v>
@@ -17527,7 +17537,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>56.7323137223528</v>
@@ -17586,7 +17596,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>60.2564702481322</v>
@@ -17645,7 +17655,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>58.9666579889489</v>
@@ -17704,7 +17714,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>57.4960164929809</v>
@@ -17763,7 +17773,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>51.6538096714813</v>
@@ -17822,7 +17832,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>53.8895953452069</v>
@@ -17881,7 +17891,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>53.7533870435689</v>
@@ -17940,7 +17950,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>70.1622697996373</v>
@@ -17999,7 +18009,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>52.6803364620866</v>
@@ -18058,7 +18068,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>49.9770898897128</v>
@@ -18117,7 +18127,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>55.5674259414808</v>
@@ -18176,7 +18186,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>51.4623262382269</v>
@@ -18235,7 +18245,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>51.5707316261091</v>
@@ -18294,7 +18304,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>56.9438094746549</v>
@@ -18353,7 +18363,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>52.6208632837869</v>
@@ -18412,7 +18422,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>54.6682855393767</v>
@@ -18471,7 +18481,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>49.3477586758045</v>
@@ -18530,7 +18540,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>54.6806788942866</v>
@@ -18589,7 +18599,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>53.991698056126</v>
@@ -18648,7 +18658,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>65.0455709887127</v>
@@ -18707,7 +18717,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>51.8521207659433</v>
@@ -18766,7 +18776,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>52.6917078593109</v>
@@ -18825,7 +18835,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>58.3128890439052</v>
@@ -18884,7 +18894,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>48.1459085039199</v>
@@ -18943,7 +18953,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>51.4963561905688</v>
@@ -19002,7 +19012,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>51.7955868849164</v>
@@ -19061,7 +19071,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>54.1517198376399</v>
@@ -19120,7 +19130,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>51.906711832319</v>
@@ -19179,7 +19189,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>48.3510386597211</v>
@@ -19238,7 +19248,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>53.518144384023</v>
@@ -19297,7 +19307,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>53.0344836217304</v>
@@ -19356,7 +19366,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>65.7863003996706</v>
@@ -19415,7 +19425,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>52.0937177436956</v>
@@ -19474,7 +19484,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>48.1599448536969</v>
@@ -19533,7 +19543,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>54.4481382012771</v>
@@ -19592,7 +19602,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>52.9209966510892</v>
@@ -19651,7 +19661,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>51.3173068498867</v>
@@ -19710,7 +19720,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>53.7335807332686</v>
@@ -19769,7 +19779,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>54.8658358507621</v>
@@ -19828,7 +19838,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>51.8207122625734</v>
@@ -19887,7 +19897,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>49.8559752134098</v>
@@ -19946,7 +19956,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>53.4393242387797</v>
@@ -20005,7 +20015,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>50.9771144829808</v>
@@ -20064,7 +20074,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>66.389495482528</v>
@@ -20123,7 +20133,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>51.4423543677601</v>
@@ -20182,7 +20192,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>48.707971162632</v>
@@ -20241,7 +20251,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>52.2327253689177</v>
@@ -20300,7 +20310,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>52.5174913342801</v>
@@ -20359,7 +20369,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>50.9416108386554</v>
@@ -20418,7 +20428,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>53.0454411554204</v>
@@ -20477,7 +20487,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>56.1810377282003</v>
@@ -20536,7 +20546,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>53.3421061776047</v>
@@ -20595,7 +20605,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>51.2081049538338</v>
@@ -20654,7 +20664,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>54.7389396335636</v>
@@ -20713,7 +20723,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>55.5518518360096</v>
@@ -20772,7 +20782,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>68.3964197494532</v>
@@ -20831,7 +20841,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>54.8963960306231</v>
@@ -20890,7 +20900,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>51.9132973474691</v>
@@ -20949,7 +20959,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>57.1730508071674</v>
@@ -21008,7 +21018,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>56.8817920009961</v>
@@ -21067,7 +21077,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>53.5842540555205</v>
@@ -21126,7 +21136,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>55.3966936845068</v>
@@ -21185,7 +21195,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>59.8689763554909</v>
@@ -21244,7 +21254,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>61.1879014723105</v>
@@ -21303,7 +21313,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>59.6981917955324</v>
@@ -21362,7 +21372,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>64.6945287020769</v>
@@ -21421,7 +21431,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>62.596517614141</v>
@@ -21480,7 +21490,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>78.225676206142</v>
@@ -21539,7 +21549,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>58.2099265365871</v>
@@ -21598,7 +21608,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>54.7182928024749</v>
@@ -21657,7 +21667,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>61.6467295444961</v>
@@ -21716,7 +21726,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>55.6910555032772</v>
@@ -21775,7 +21785,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>56.766976755547</v>
@@ -21834,7 +21844,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>58.0867597797523</v>
@@ -21893,7 +21903,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>57.748945336331</v>
@@ -21952,7 +21962,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>59.0577042203124</v>
@@ -22011,7 +22021,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>52.3298182807479</v>
@@ -22070,7 +22080,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>55.5944664773738</v>
@@ -22129,7 +22139,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>57.1932317600073</v>
@@ -22188,7 +22198,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>68.2156979762974</v>
@@ -22247,7 +22257,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>54.9088349707043</v>
@@ -22306,7 +22316,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>51.0974607379748</v>
@@ -22365,7 +22375,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>57.8946302863318</v>
@@ -22424,7 +22434,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>55.595930007425</v>
@@ -22483,7 +22493,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>54.7439576863762</v>
@@ -22542,7 +22552,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>55.129527488879</v>
@@ -22601,7 +22611,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>54.5116091930909</v>
@@ -22660,7 +22670,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>54.9436210092428</v>
@@ -22719,7 +22729,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>50.3775422647919</v>
@@ -22778,7 +22788,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>51.3355355589654</v>
@@ -22837,7 +22847,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>53.1205710244378</v>
@@ -22896,7 +22906,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>66.1347021607982</v>
@@ -22955,7 +22965,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>52.9697698878784</v>
@@ -23014,7 +23024,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>49.0921885816217</v>
@@ -23073,7 +23083,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>53.74760684358</v>
@@ -23132,7 +23142,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2"/>
       <c r="C353" s="3" t="n">
@@ -23165,7 +23175,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2"/>
       <c r="C354" s="3" t="n">
@@ -23198,7 +23208,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2"/>
       <c r="C355" s="3" t="n">
@@ -23231,7 +23241,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2"/>
       <c r="C356" s="3" t="n">
@@ -23264,7 +23274,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2"/>
       <c r="C357" s="3" t="n">
@@ -23297,7 +23307,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2"/>
       <c r="C358" s="3" t="n">
@@ -23330,7 +23340,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2"/>
       <c r="C359" s="3" t="n">
@@ -23363,7 +23373,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2"/>
       <c r="C360" s="3" t="n">
@@ -23396,7 +23406,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2"/>
       <c r="C361" s="3" t="n">
@@ -23429,7 +23439,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2"/>
       <c r="C362" s="3" t="n">
@@ -23462,7 +23472,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2"/>
       <c r="C363" s="3" t="n">
@@ -23495,7 +23505,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2"/>
       <c r="C364" s="3" t="n">
@@ -23528,7 +23538,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2"/>
       <c r="C365" s="3"/>
@@ -23551,7 +23561,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2"/>
       <c r="C366" s="3"/>
@@ -23574,7 +23584,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2"/>
       <c r="C367" s="3"/>
@@ -23597,7 +23607,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2"/>
       <c r="C368" s="3"/>
@@ -23620,7 +23630,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2"/>
       <c r="C369" s="3"/>
@@ -23643,7 +23653,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2"/>
       <c r="C370" s="3"/>
@@ -23666,7 +23676,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2"/>
       <c r="C371" s="3"/>
@@ -23689,7 +23699,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2"/>
       <c r="C372" s="3"/>
@@ -23712,7 +23722,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2"/>
       <c r="C373" s="3"/>
@@ -23735,7 +23745,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2"/>
       <c r="C374" s="3"/>
@@ -23758,7 +23768,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2"/>
       <c r="C375" s="3"/>
@@ -23781,7 +23791,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2"/>
       <c r="C376" s="3"/>
@@ -23804,7 +23814,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2"/>
       <c r="C377" s="3"/>
@@ -23827,7 +23837,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2"/>
       <c r="C378" s="3"/>
@@ -23850,7 +23860,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2"/>
       <c r="C379" s="3"/>
@@ -23873,7 +23883,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2"/>
       <c r="C380" s="3"/>
@@ -23896,7 +23906,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2"/>
       <c r="C381" s="3"/>
@@ -23919,7 +23929,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2"/>
       <c r="C382" s="3"/>
@@ -23942,7 +23952,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2"/>
       <c r="C383" s="3"/>
@@ -23965,7 +23975,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2"/>
       <c r="C384" s="3"/>
@@ -23988,7 +23998,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2"/>
       <c r="C385" s="3"/>
@@ -24011,7 +24021,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2"/>
       <c r="C386" s="3"/>
@@ -24034,7 +24044,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2"/>
       <c r="C387" s="3"/>
@@ -24057,7 +24067,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2"/>
       <c r="C388" s="3"/>
@@ -24080,7 +24090,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2"/>
       <c r="C389" s="3"/>
@@ -24103,7 +24113,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3"/>
@@ -24126,7 +24136,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3"/>
@@ -24149,7 +24159,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3"/>
@@ -24172,7 +24182,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3"/>
@@ -24195,7 +24205,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3"/>
@@ -24218,7 +24228,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3"/>
@@ -24241,7 +24251,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3"/>
@@ -24264,7 +24274,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3"/>
@@ -24287,7 +24297,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3"/>
@@ -24310,7 +24320,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3"/>
@@ -24333,7 +24343,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3"/>
@@ -24356,7 +24366,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3"/>
@@ -24379,7 +24389,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -24402,7 +24412,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -24425,7 +24435,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -24448,7 +24458,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -24471,7 +24481,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -24494,7 +24504,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -24517,7 +24527,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -24540,7 +24550,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -24574,97 +24584,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
   </sheetData>
@@ -24688,7 +24698,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -24698,160 +24708,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0185568330535138</v>
+        <v>-0.0182142315646441</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.00061200369648616</v>
+        <v>-0.000332305048471</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0209696713615437</v>
+        <v>0.0193887760482077</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0598954505221596</v>
+        <v>0.0576047517752578</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.0851178356036261</v>
+        <v>0.0828738460456294</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.110714179512468</v>
+        <v>0.109195094994012</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.169762164206358</v>
+        <v>0.168654653837187</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.24185920879637</v>
+        <v>0.240968903248353</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.3320134621667</v>
+        <v>0.331074496546127</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.435319377953837</v>
+        <v>0.433700046183411</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.470778581408282</v>
+        <v>0.468768245511086</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.461655478973808</v>
+        <v>0.460270878317805</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.471332904617273</v>
+        <v>0.471076351264492</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.478481700729284</v>
+        <v>0.478830125154761</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.473767582855067</v>
+        <v>0.47420255963667</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.453598143044007</v>
+        <v>0.454339446240957</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.425370518017448</v>
+        <v>0.425932052315121</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.416001426370137</v>
+        <v>0.415961598407947</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.382630418645754</v>
+        <v>0.382396534293613</v>
       </c>
     </row>
     <row r="24">

</xml_diff>